<commit_message>
airports parquet file do not drop na because some rows might be lost
</commit_message>
<xml_diff>
--- a/Documents/History of versions.xlsx
+++ b/Documents/History of versions.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\git\PRCdataChallenge2025\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F716FFFA-3037-4D55-99F1-4FB9D8600085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{268A9CD6-B372-4CC1-B899-FADEF0EF1A29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="2790" windowWidth="29040" windowHeight="15720" xr2:uid="{8278A78D-C433-40FD-A6EF-2CA63E3DF70B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{8278A78D-C433-40FD-A6EF-2CA63E3DF70B}"/>
   </bookViews>
   <sheets>
     <sheet name="Submissions versions" sheetId="1" r:id="rId1"/>
+    <sheet name="v16 errors" sheetId="2" r:id="rId2"/>
+    <sheet name="missing airport " sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="57">
   <si>
     <t>date</t>
   </si>
@@ -111,13 +113,109 @@
   </si>
   <si>
     <t>probably not the same list of capped columns</t>
+  </si>
+  <si>
+    <t>v15</t>
+  </si>
+  <si>
+    <t>add distance Nm from origin to each fuel position and from each fuel position to destination</t>
+  </si>
+  <si>
+    <t>error missing records not reaching 24288 records</t>
+  </si>
+  <si>
+    <t xml:space="preserve">error records with no predictions see flight </t>
+  </si>
+  <si>
+    <t>v16</t>
+  </si>
+  <si>
+    <t>prc811832834</t>
+  </si>
+  <si>
+    <t>2025-09-21 13:50:14.198</t>
+  </si>
+  <si>
+    <t>2025-09-21 13:51:35.265</t>
+  </si>
+  <si>
+    <t>2025-09-21 14:03:45.109</t>
+  </si>
+  <si>
+    <t>2025-09-21 14:05:47.389</t>
+  </si>
+  <si>
+    <t>2025-09-21 14:08:48.209</t>
+  </si>
+  <si>
+    <t>2025-09-21 14:09:47.685</t>
+  </si>
+  <si>
+    <t>2025-09-21 14:10:48.612</t>
+  </si>
+  <si>
+    <t>2025-09-21 14:16:55.199</t>
+  </si>
+  <si>
+    <t>2025-09-21 14:20:56.774</t>
+  </si>
+  <si>
+    <t>2025-09-21 14:21:53.69</t>
+  </si>
+  <si>
+    <t>2025-09-21 14:22:55.215</t>
+  </si>
+  <si>
+    <t>2025-09-21 14:23:55.715</t>
+  </si>
+  <si>
+    <t>2025-09-21 14:24:55.618</t>
+  </si>
+  <si>
+    <t>2025-09-21 14:26:56.363</t>
+  </si>
+  <si>
+    <t>idx</t>
+  </si>
+  <si>
+    <t>flight_id</t>
+  </si>
+  <si>
+    <t>start</t>
+  </si>
+  <si>
+    <t>end</t>
+  </si>
+  <si>
+    <t>fuel_kg</t>
+  </si>
+  <si>
+    <t>origin_longitude_deg 24255 non-null float64</t>
+  </si>
+  <si>
+    <t>54 origin_latitude_deg 24255 non-null float64</t>
+  </si>
+  <si>
+    <t>55 origin_elevation_ft 24255 non-null float64</t>
+  </si>
+  <si>
+    <t>56 destination_longitude_deg 24255 non-null float64</t>
+  </si>
+  <si>
+    <t>57 destination_latitude_deg 24255 non-null float64</t>
+  </si>
+  <si>
+    <t>58 destination_elevation_ft 24255 non-null float64</t>
+  </si>
+  <si>
+    <t>should have 24289 values</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -139,6 +237,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -154,7 +258,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -201,11 +305,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -214,6 +329,13 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -548,11 +670,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4734075F-58FB-48FD-9239-DDB8EC5D04CD}">
-  <dimension ref="A3:E10"/>
+  <dimension ref="A3:E12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="49.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="65.36328125" customWidth="1"/>
     <col min="4" max="4" width="22.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -674,8 +796,251 @@
         <v>24</v>
       </c>
     </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="3">
+        <v>45962</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" s="3">
+        <v>45963</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59FB7211-334C-4DF3-AC1A-60225B95E2E2}">
+  <dimension ref="A2:E12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.08984375" customWidth="1"/>
+    <col min="2" max="2" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="9">
+        <v>19489</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" s="9"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="9">
+        <v>19490</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="9"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="9">
+        <v>19491</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="9"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="9">
+        <v>19492</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" s="9"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="9">
+        <v>19493</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="9"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="9">
+        <v>19494</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" s="9"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" s="9">
+        <v>19495</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="9"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="9">
+        <v>19496</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="E11" s="9"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" s="9">
+        <v>19497</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="E12" s="9"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20A8F210-0A7E-4A60-8FF2-8DA00254F968}">
+  <dimension ref="A4:K9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="K4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="10" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="10" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
version v20 clean outliers on both train and ranking with limited list of columns to clen
</commit_message>
<xml_diff>
--- a/Documents/History of versions.xlsx
+++ b/Documents/History of versions.xlsx
@@ -8,14 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\git\PRCdataChallenge2025\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{268A9CD6-B372-4CC1-B899-FADEF0EF1A29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{204B8732-423B-44C0-9094-5D4B743661E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{8278A78D-C433-40FD-A6EF-2CA63E3DF70B}"/>
+    <workbookView xWindow="38280" yWindow="2790" windowWidth="29040" windowHeight="15720" xr2:uid="{8278A78D-C433-40FD-A6EF-2CA63E3DF70B}"/>
   </bookViews>
   <sheets>
     <sheet name="Submissions versions" sheetId="1" r:id="rId1"/>
     <sheet name="v16 errors" sheetId="2" r:id="rId2"/>
-    <sheet name="missing airport " sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="62">
   <si>
     <t>date</t>
   </si>
@@ -190,32 +189,47 @@
     <t>fuel_kg</t>
   </si>
   <si>
-    <t>origin_longitude_deg 24255 non-null float64</t>
-  </si>
-  <si>
-    <t>54 origin_latitude_deg 24255 non-null float64</t>
-  </si>
-  <si>
-    <t>55 origin_elevation_ft 24255 non-null float64</t>
-  </si>
-  <si>
-    <t>56 destination_longitude_deg 24255 non-null float64</t>
-  </si>
-  <si>
-    <t>57 destination_latitude_deg 24255 non-null float64</t>
-  </si>
-  <si>
-    <t>58 destination_elevation_ft 24255 non-null float64</t>
-  </si>
-  <si>
-    <t>should have 24289 values</t>
+    <t>v17</t>
+  </si>
+  <si>
+    <t>361.9855</t>
+  </si>
+  <si>
+    <t>distance between origin and aircraft position at fuel start and fuel end is computed without the airport elevation</t>
+  </si>
+  <si>
+    <t>outliers capping is done on Train only and with a groupby on the aircraft code</t>
+  </si>
+  <si>
+    <t>v18</t>
+  </si>
+  <si>
+    <t>545.1602</t>
+  </si>
+  <si>
+    <t>v19</t>
+  </si>
+  <si>
+    <t>outliers capping is done on train only, capping is using stats for one column and the whole train dataset</t>
+  </si>
+  <si>
+    <t>381.4168</t>
+  </si>
+  <si>
+    <t>outliers capping is done on train and on rank also</t>
+  </si>
+  <si>
+    <t>v20</t>
+  </si>
+  <si>
+    <t>348.5089</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -237,12 +251,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Courier New"/>
-      <family val="3"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -258,7 +266,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -316,11 +324,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -333,9 +361,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -670,11 +698,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4734075F-58FB-48FD-9239-DDB8EC5D04CD}">
-  <dimension ref="A3:E12"/>
+  <dimension ref="A3:E16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="65.36328125" customWidth="1"/>
+    <col min="3" max="3" width="90.90625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -817,8 +845,65 @@
       <c r="B12" s="2" t="s">
         <v>29</v>
       </c>
+      <c r="C12" s="2"/>
       <c r="D12" s="8" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" s="3">
+        <v>45963</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" s="3">
+        <v>45963</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" s="3">
+        <v>45963</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" s="3">
+        <v>45963</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1000,47 +1085,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20A8F210-0A7E-4A60-8FF2-8DA00254F968}">
-  <dimension ref="A4:K9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="K4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="10" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="10" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="10" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="10" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="10" t="s">
-        <v>55</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
comparison of values versus epsilon
</commit_message>
<xml_diff>
--- a/Documents/History of versions.xlsx
+++ b/Documents/History of versions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\git\PRCdataChallenge2025\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{204B8732-423B-44C0-9094-5D4B743661E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82135D93-83E3-434C-90E5-7A965158D60F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="2790" windowWidth="29040" windowHeight="15720" xr2:uid="{8278A78D-C433-40FD-A6EF-2CA63E3DF70B}"/>
+    <workbookView xWindow="38280" yWindow="2790" windowWidth="29040" windowHeight="15720" tabRatio="320" xr2:uid="{8278A78D-C433-40FD-A6EF-2CA63E3DF70B}"/>
   </bookViews>
   <sheets>
     <sheet name="Submissions versions" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="71">
   <si>
     <t>date</t>
   </si>
@@ -223,6 +223,33 @@
   </si>
   <si>
     <t>348.5089</t>
+  </si>
+  <si>
+    <t>v21</t>
+  </si>
+  <si>
+    <t>add TAS and CAS at fuel start and fuel end computed from mach</t>
+  </si>
+  <si>
+    <t>286.9913</t>
+  </si>
+  <si>
+    <t>326.0406</t>
+  </si>
+  <si>
+    <t>v22</t>
+  </si>
+  <si>
+    <t>v23</t>
+  </si>
+  <si>
+    <t>352.4399</t>
+  </si>
+  <si>
+    <t>correct the time delta to zero for burn start and end versus takeoff and landed</t>
+  </si>
+  <si>
+    <t>epochs 200 instead of 150</t>
   </si>
 </sst>
 </file>
@@ -266,7 +293,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -344,11 +371,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -363,7 +401,8 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -698,7 +737,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4734075F-58FB-48FD-9239-DDB8EC5D04CD}">
-  <dimension ref="A3:E16"/>
+  <dimension ref="A3:E19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.08984375" style="1" bestFit="1" customWidth="1"/>
@@ -758,7 +797,7 @@
       <c r="C6" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E6" t="s">
@@ -904,6 +943,48 @@
       </c>
       <c r="D16" s="7" t="s">
         <v>61</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" s="1">
+        <v>45964</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" s="1">
+        <v>45964</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" s="1">
+        <v>45964</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
re re organize base class
</commit_message>
<xml_diff>
--- a/Documents/History of versions.xlsx
+++ b/Documents/History of versions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\git\PRCdataChallenge2025\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82135D93-83E3-434C-90E5-7A965158D60F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C310C3E-A635-43F7-BE2E-A8902EBE7035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="2790" windowWidth="29040" windowHeight="15720" tabRatio="320" xr2:uid="{8278A78D-C433-40FD-A6EF-2CA63E3DF70B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="320" xr2:uid="{8278A78D-C433-40FD-A6EF-2CA63E3DF70B}"/>
   </bookViews>
   <sheets>
     <sheet name="Submissions versions" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="83">
   <si>
     <t>date</t>
   </si>
@@ -228,9 +228,6 @@
     <t>v21</t>
   </si>
   <si>
-    <t>add TAS and CAS at fuel start and fuel end computed from mach</t>
-  </si>
-  <si>
     <t>286.9913</t>
   </si>
   <si>
@@ -250,6 +247,45 @@
   </si>
   <si>
     <t>epochs 200 instead of 150</t>
+  </si>
+  <si>
+    <t>v24</t>
+  </si>
+  <si>
+    <t>414.6309</t>
+  </si>
+  <si>
+    <t>extended features , many missing, mean absolute error, epochs 300, get dummies on the aircraft type</t>
+  </si>
+  <si>
+    <t>v25</t>
+  </si>
+  <si>
+    <t>use rmse , epochs still 300</t>
+  </si>
+  <si>
+    <t>417.5815</t>
+  </si>
+  <si>
+    <t>436.7149</t>
+  </si>
+  <si>
+    <t>epoch 200 , loss = rmse , dummies suppressed</t>
+  </si>
+  <si>
+    <t>v26</t>
+  </si>
+  <si>
+    <t>epoch = 300 , dummies used again, compute TAS and CAS from mach in any case without conditions</t>
+  </si>
+  <si>
+    <t>v27</t>
+  </si>
+  <si>
+    <t>426.4757</t>
+  </si>
+  <si>
+    <t>add TAS and CAS at fuel start and fuel end computed from mach when TAS and CAS are missing</t>
   </si>
 </sst>
 </file>
@@ -293,7 +329,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -376,6 +412,19 @@
         <color indexed="64"/>
       </left>
       <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -402,7 +451,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -737,7 +786,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4734075F-58FB-48FD-9239-DDB8EC5D04CD}">
-  <dimension ref="A3:E19"/>
+  <dimension ref="A3:E23"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.08984375" style="1" bestFit="1" customWidth="1"/>
@@ -953,10 +1002,10 @@
         <v>62</v>
       </c>
       <c r="C17" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>63</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
@@ -964,27 +1013,83 @@
         <v>45964</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
         <v>45964</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="D19" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="C19" s="13" t="s">
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" s="3">
+        <v>45967</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>68</v>
+      <c r="C20" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" s="3">
+        <v>45967</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" s="3">
+        <v>45967</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" s="3">
+        <v>45967</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D23" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v28 - rmse = 291
</commit_message>
<xml_diff>
--- a/Documents/History of versions.xlsx
+++ b/Documents/History of versions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\git\PRCdataChallenge2025\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C310C3E-A635-43F7-BE2E-A8902EBE7035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78D5B1AA-628C-4E1F-BDB5-00BB86198BCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="320" xr2:uid="{8278A78D-C433-40FD-A6EF-2CA63E3DF70B}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="86">
   <si>
     <t>date</t>
   </si>
@@ -286,6 +286,15 @@
   </si>
   <si>
     <t>add TAS and CAS at fuel start and fuel end computed from mach when TAS and CAS are missing</t>
+  </si>
+  <si>
+    <t>v28</t>
+  </si>
+  <si>
+    <t>epoch 200 , TAS and CAS computed from mach with python aerocalc</t>
+  </si>
+  <si>
+    <t>291.6856</t>
   </si>
 </sst>
 </file>
@@ -435,7 +444,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -452,6 +461,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -786,7 +796,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4734075F-58FB-48FD-9239-DDB8EC5D04CD}">
-  <dimension ref="A3:E23"/>
+  <dimension ref="A3:E24"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.08984375" style="1" bestFit="1" customWidth="1"/>
@@ -1090,6 +1100,20 @@
       </c>
       <c r="D23" t="s">
         <v>81</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" s="1">
+        <v>45970</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="D24" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
create interpolated flights data files
</commit_message>
<xml_diff>
--- a/Documents/History of versions.xlsx
+++ b/Documents/History of versions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\git\PRCdataChallenge2025\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78D5B1AA-628C-4E1F-BDB5-00BB86198BCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B3EFFE4-F5D3-4CC8-946B-1CFDAB1039A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="320" xr2:uid="{8278A78D-C433-40FD-A6EF-2CA63E3DF70B}"/>
   </bookViews>
@@ -291,10 +291,10 @@
     <t>v28</t>
   </si>
   <si>
-    <t>epoch 200 , TAS and CAS computed from mach with python aerocalc</t>
-  </si>
-  <si>
     <t>291.6856</t>
+  </si>
+  <si>
+    <t>epoch 200 , TAS and CAS computed from mach with python aerocalc, zscore cleaning of train records</t>
   </si>
 </sst>
 </file>
@@ -444,7 +444,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -461,7 +461,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1095,10 +1094,10 @@
       <c r="B23" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="2" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1109,11 +1108,11 @@
       <c r="B24" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C24" s="14" t="s">
+      <c r="C24" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="D24" t="s">
-        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
prepare for flight interpolation
</commit_message>
<xml_diff>
--- a/Documents/History of versions.xlsx
+++ b/Documents/History of versions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\git\PRCdataChallenge2025\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B3EFFE4-F5D3-4CC8-946B-1CFDAB1039A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8E61F3D-1973-48CB-B6FC-5FEBF72E6B61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="320" xr2:uid="{8278A78D-C433-40FD-A6EF-2CA63E3DF70B}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="88">
   <si>
     <t>date</t>
   </si>
@@ -295,6 +295,12 @@
   </si>
   <si>
     <t>epoch 200 , TAS and CAS computed from mach with python aerocalc, zscore cleaning of train records</t>
+  </si>
+  <si>
+    <t>v29</t>
+  </si>
+  <si>
+    <t>new final fuel input</t>
   </si>
 </sst>
 </file>
@@ -444,7 +450,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -461,6 +467,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -795,7 +802,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4734075F-58FB-48FD-9239-DDB8EC5D04CD}">
-  <dimension ref="A3:E24"/>
+  <dimension ref="A3:E25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.08984375" style="1" bestFit="1" customWidth="1"/>
@@ -1111,8 +1118,16 @@
       <c r="C24" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D24" s="5" t="s">
         <v>84</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B25" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C25" s="14" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
history of versions v29
</commit_message>
<xml_diff>
--- a/Documents/History of versions.xlsx
+++ b/Documents/History of versions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\git\PRCdataChallenge2025\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8E61F3D-1973-48CB-B6FC-5FEBF72E6B61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F9268DC-A99F-42DE-B3FA-6502E1B390C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="320" xr2:uid="{8278A78D-C433-40FD-A6EF-2CA63E3DF70B}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="89">
   <si>
     <t>date</t>
   </si>
@@ -300,7 +300,10 @@
     <t>v29</t>
   </si>
   <si>
-    <t>new final fuel input</t>
+    <t>epoch = 200, new final fuel input , TAS and CAS computed in the java part</t>
+  </si>
+  <si>
+    <t>328.9957</t>
   </si>
 </sst>
 </file>
@@ -344,7 +347,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -446,11 +449,42 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -467,7 +501,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1109,7 +1145,7 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A24" s="1">
+      <c r="A24" s="14">
         <v>45970</v>
       </c>
       <c r="B24" s="2" t="s">
@@ -1123,11 +1159,17 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B25" s="14" t="s">
+      <c r="A25" s="15">
+        <v>45977</v>
+      </c>
+      <c r="B25" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="C25" s="14" t="s">
+      <c r="C25" s="2" t="s">
         <v>87</v>
+      </c>
+      <c r="D25" t="s">
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
prepare for rebuild some flight with openap
</commit_message>
<xml_diff>
--- a/Documents/History of versions.xlsx
+++ b/Documents/History of versions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\git\PRCdataChallenge2025\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C74292C6-10FA-4418-A0B4-79AAFD316C00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9035CBE3-C993-489F-99DE-E66FE0223684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="320" xr2:uid="{8278A78D-C433-40FD-A6EF-2CA63E3DF70B}"/>
   </bookViews>
@@ -7600,7 +7600,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -7638,7 +7638,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8485,7 +8484,7 @@
       <c r="B38" s="12" t="s">
         <v>2447</v>
       </c>
-      <c r="C38" s="27" t="s">
+      <c r="C38" s="26" t="s">
         <v>2448</v>
       </c>
       <c r="D38" t="s">

</xml_diff>

<commit_message>
compute flight data using openap
</commit_message>
<xml_diff>
--- a/Documents/History of versions.xlsx
+++ b/Documents/History of versions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\git\PRCdataChallenge2025\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{672107C4-A747-42A6-8F0C-A7384E35F549}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CDFB28C-E327-4267-A495-A068D732F7F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="320" xr2:uid="{8278A78D-C433-40FD-A6EF-2CA63E3DF70B}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2467" uniqueCount="2452">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2470" uniqueCount="2455">
   <si>
     <t>date</t>
   </si>
@@ -7394,6 +7394,15 @@
   </si>
   <si>
     <t>v43</t>
+  </si>
+  <si>
+    <t>518.3411</t>
+  </si>
+  <si>
+    <t>v44</t>
+  </si>
+  <si>
+    <t>compute a full trajectory for Rank file prc812317830</t>
   </si>
 </sst>
 </file>
@@ -7982,7 +7991,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4734075F-58FB-48FD-9239-DDB8EC5D04CD}">
-  <dimension ref="A3:E41"/>
+  <dimension ref="A3:E44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.85546875" style="1" customWidth="1"/>
@@ -8508,7 +8517,7 @@
       <c r="B39" s="2" t="s">
         <v>2451</v>
       </c>
-      <c r="C39" s="27" t="s">
+      <c r="C39" s="26" t="s">
         <v>2449</v>
       </c>
       <c r="D39" t="s">
@@ -8516,12 +8525,26 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C40" s="26" t="s">
+      <c r="A40" s="1">
+        <v>45985</v>
+      </c>
+      <c r="B40" s="15" t="s">
+        <v>2453</v>
+      </c>
+      <c r="C40" s="27" t="s">
+        <v>2454</v>
+      </c>
+      <c r="D40" t="s">
+        <v>2452</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C43" s="26" t="s">
         <v>2439</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C41" s="26" t="s">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C44" s="26" t="s">
         <v>2440</v>
       </c>
     </row>

</xml_diff>